<commit_message>
Added note on other traces
</commit_message>
<xml_diff>
--- a/board/v0_1/production_files/Required_impedance_control.xlsx
+++ b/board/v0_1/production_files/Required_impedance_control.xlsx
@@ -1659,7 +1659,23 @@
       <c r="H2" s="11" t="n"/>
       <c r="I2" s="13" t="inlineStr">
         <is>
-          <t>Ethernet, PCIe, PCIe refclk, USB2: USBD_P/USBD_N, PCIE.REFCLK_P/REFCLK_N, PCISLOT.TX_P/TX_N, PCIE.TX_P/TX_N, PCIE.RX_P/RX_N, RJTX_P/RJTX_N, RJRX_P/RJRX_N</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00C00000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">NOTE: applies ONLY to coupled differential pairs (6 mil width, 6 mil spacing). Single 6 mil traces on this layer are NOT impedance controlled - do not adjust them.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Ethernet, PCIe, PCIe refclk, USB2: USBD_P/USBD_N, PCIE.REFCLK_P/REFCLK_N, PCISLOT.TX_P/TX_N, PCIE.TX_P/TX_N, PCIE.RX_P/RX_N, RJTX_P/RJTX_N, RJRX_P/RJRX_N</t>
+          </r>
         </is>
       </c>
     </row>
@@ -2047,7 +2063,23 @@
       <c r="H14" s="11" t="n"/>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>PCIe, PCIe refclk: REFCLKAC_P/REFCLKAC_N, PCIE.RX_P/RX_N</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="00C00000"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">NOTE: applies ONLY to coupled differential pairs (6 mil width, 6 mil spacing). Single 6 mil traces on this layer are NOT impedance controlled - do not adjust them.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t>PCIe, PCIe refclk: REFCLKAC_P/REFCLKAC_N, PCIE.RX_P/RX_N</t>
+          </r>
         </is>
       </c>
     </row>

</xml_diff>